<commit_message>
chore: save local outputs and log files
</commit_message>
<xml_diff>
--- a/output/abb_report.xlsx
+++ b/output/abb_report.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ABB Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ABB Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -88,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -102,9 +102,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -475,7 +472,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,7 +502,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>1519768.5</v>
+        <v>144014448.9</v>
       </c>
     </row>
     <row r="5">
@@ -514,8 +511,10 @@
           <t>Average 3 Months ABB</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
-        <v>658796.6</v>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Data Unavailable</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -524,8 +523,10 @@
           <t>Average 6 Months ABB</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>507120.81</v>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Data Unavailable</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>